<commit_message>
feat: programas academicos y asignaturas con codigo autogenerado en el backend
</commit_message>
<xml_diff>
--- a/backend/pruebas/plantilla-estudiantes.xlsx
+++ b/backend/pruebas/plantilla-estudiantes.xlsx
@@ -78,11 +78,6 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nombreAsignatura</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
           <t xml:space="preserve">grupo</t>
         </is>
       </c>
@@ -135,7 +130,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingenieria de Sistemas</t>
+          <t xml:space="preserve">Ingeniería de Sistemas</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -150,15 +145,10 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SIS101</t>
+          <t xml:space="preserve">ISI-001</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Introduccion a la Informatica</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -212,7 +202,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingenieria de Sistemas</t>
+          <t xml:space="preserve">Ingeniería de Sistemas</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -227,15 +217,10 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SIS102</t>
+          <t xml:space="preserve">ISI-002</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Programacion Orientada a Objetos</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -289,7 +274,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingenieria Electronica</t>
+          <t xml:space="preserve">Ingeniería Electrónica y Telecomunicaciones</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -304,15 +289,10 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ELE201</t>
+          <t xml:space="preserve">IET-001</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Circuitos Electricos</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>

</xml_diff>

<commit_message>
T12.1: cargo en vez de dependencia, facultad FIET fija, edición completa de estudiante y funcionario, situaciones R0-R3, faltas y nota como texto, observaciones del Decano opcionales y ocultas al estudiante, mensaje de respuesta al estudiante
</commit_message>
<xml_diff>
--- a/backend/pruebas/plantilla-estudiantes.xlsx
+++ b/backend/pruebas/plantilla-estudiantes.xlsx
@@ -68,15 +68,10 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t xml:space="preserve">facultad</t>
+          <t xml:space="preserve">codigoAsignatura</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">codigoAsignatura</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t xml:space="preserve">grupo</t>
         </is>
@@ -140,15 +135,10 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIET</t>
+          <t xml:space="preserve">ISI-001</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ISI-001</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -212,15 +202,10 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIET</t>
+          <t xml:space="preserve">ISI-002</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ISI-002</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -284,15 +269,10 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIET</t>
+          <t xml:space="preserve">IET-001</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IET-001</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>

</xml_diff>